<commit_message>
Improve instrument extraction coverage
</commit_message>
<xml_diff>
--- a/outputs/instrument_only.xlsx
+++ b/outputs/instrument_only.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,30 +468,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>6820-R2-67001-03_NOHD-NI01_1..pdf</t>
+          <t>6820-R2-61029-01_WWXL-FP01_1..pdf</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>6820-R2-67001-03</t>
+          <t>6820-R2-61029-01</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>14-LV-68250</t>
+          <t>14-FO-68989</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>14-LV-68250</t>
+          <t>14-FO-68989</t>
         </is>
       </c>
       <c r="G2" t="n">
@@ -501,16 +501,16 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>6820-R2-67001-06_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67001-03_NOHD-NI01_1..pdf</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>6820-R2-67001-06</t>
+          <t>6820-R2-67001-03</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -519,12 +519,12 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>14-FO-68109</t>
+          <t>14-LV-68250</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>14-FO-68109</t>
+          <t>14-LV-68250</t>
         </is>
       </c>
       <c r="G3" t="n">
@@ -534,12 +534,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>6820-R2-67073-02_NOHD-SS01_0.pdf</t>
+          <t>6820-R2-67001-06_NOHD-NI01_0..pdf</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6820-R2-67073-02</t>
+          <t>6820-R2-67001-06</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -547,17 +547,17 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>14-HV-68460</t>
+          <t>14-FO-68109</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>14-HV-68460</t>
+          <t>14-FO-68109</t>
         </is>
       </c>
       <c r="G4" t="n">
@@ -567,30 +567,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>6820-R2-67080-01_SCXL-CS02_1..pdf</t>
+          <t>6820-R2-67008-03_EPCW-CS01_1..pdf</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>6820-R2-67080-01</t>
+          <t>6820-R2-67008-03</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>14-HV-68520</t>
+          <t>14-TI-68419</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>14-HV-68520</t>
+          <t>14-TI-68419</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -600,30 +600,30 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>6820-R2-67093-02_NOHD-SS01_1.pdf</t>
+          <t>6820-R2-67018-02_SCXL-CS02_0..pdf</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>6820-R2-67093-02</t>
+          <t>6820-R2-67018-02</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>14-FIT-68160</t>
+          <t>14-PI-68759</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>14-FIT-68160</t>
+          <t>14-PI-68759</t>
         </is>
       </c>
       <c r="G6" t="n">
@@ -633,30 +633,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>6820-R2-67093-04_NOHD-SS01_0.pdf</t>
+          <t>6820-R2-67021-05_NOHD-NI03_1..pdf</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>6820-R2-67093-04</t>
+          <t>6820-R2-67021-05</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>14-LV-68270</t>
+          <t>14-PI-68789</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>14-LV-68270</t>
+          <t>14-PI-68789</t>
         </is>
       </c>
       <c r="G7" t="n">
@@ -666,30 +666,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>6820-R2-67111-03_EPCW-CS01_0..pdf</t>
+          <t>6820-R2-67022-12_NOHD-NI03_1..pdf</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>6820-R2-67111-03</t>
+          <t>6820-R2-67022-12</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>14-PV-68353</t>
+          <t>14-PI-68779</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>14-PV-68353</t>
+          <t>14-PI-68779</t>
         </is>
       </c>
       <c r="G8" t="n">
@@ -699,30 +699,30 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>6820-R2-67125-04_NOHD-SS01_0..pdf</t>
+          <t>6820-R2-67040-03_NOHD-NI01_1..pdf</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>6820-R2-67125-04</t>
+          <t>6820-R2-67040-03</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>14-FE-68180</t>
+          <t>14-TI-68429</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14-FE-68180</t>
+          <t>14-TI-68429</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -732,30 +732,30 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>6820-R2-67125-05_NOHD-SS01_1.pdf</t>
+          <t>6820-R2-67040-06_NOHD-NI01_0..pdf</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>6820-R2-67125-05</t>
+          <t>6820-R2-67040-06</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>14-FV-68180</t>
+          <t>14-LV-68240</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>14-FV-68180</t>
+          <t>14-LV-68240</t>
         </is>
       </c>
       <c r="G10" t="n">
@@ -765,30 +765,30 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>6820-R2-67129-06_EPCL-SS01_1.pdf</t>
+          <t>6820-R2-67040-10_NOHD-NI01_0..pdf</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>6820-R2-67129-06</t>
+          <t>6820-R2-67040-10</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>14-PI-68829</t>
+          <t>14-TE-68431</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>14-PI-68829</t>
+          <t>14-TE-68431</t>
         </is>
       </c>
       <c r="G11" t="n">
@@ -798,30 +798,30 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>6820-R2-67130-09_EPCL-SS01_1.pdf</t>
+          <t>6820-R2-67044-01_SCXL-CS02_1..pdf</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>6820-R2-67130-09</t>
+          <t>6820-R2-67044-01</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>14-PI-68819</t>
+          <t>14-TI-68439</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>14-PI-68819</t>
+          <t>14-TI-68439</t>
         </is>
       </c>
       <c r="G12" t="n">
@@ -831,30 +831,30 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>6820-R2-67133-02_EPCL-SS01_0..pdf</t>
+          <t>6820-R2-67044-05_SCXL-CS02_1..pdf</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>6820-R2-67133-02</t>
+          <t>6820-R2-67044-05</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>14-AE-68090</t>
+          <t>14-TE-68480</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>14-AE-68090</t>
+          <t>14-TE-68480</t>
         </is>
       </c>
       <c r="G13" t="n">
@@ -864,30 +864,30 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>6820-R2-67134-03_EPCL-SS01_0..pdf</t>
+          <t>6820-R2-67055-02_EPCL-SS01_1..pdf</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>6820-R2-67134-03</t>
+          <t>6820-R2-67055-02</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>14-FI-68119</t>
+          <t>14-FO-68149</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>14-FI-68119</t>
+          <t>14-FO-68149</t>
         </is>
       </c>
       <c r="G14" t="n">
@@ -897,30 +897,30 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6820-R2-67143-01_NOHD-SS01_0..pdf</t>
+          <t>6820-R2-67065-05_NOHD-NI01_1..pdf</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>6820-R2-67143-01</t>
+          <t>6820-R2-67065-05</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>14-PIT-68353</t>
+          <t>14-TE-68459</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>14-PIT-68353</t>
+          <t>14-TE-68459</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -930,30 +930,30 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>6820-R2-67164-02_CTWL-CS01_2.pdf</t>
+          <t>6820-R2-67065-07_NOHD-NI01_2..pdf</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6820-R2-67164-02</t>
+          <t>6820-R2-67065-07</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>14-FE-68170</t>
+          <t>14-TE-68432</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>14-FE-68170</t>
+          <t>14-TE-68432</t>
         </is>
       </c>
       <c r="G16" t="n">
@@ -963,30 +963,30 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>6820-R2-67181-05_SLPG-CS01_0..pdf</t>
+          <t>6820-R2-67065-07_NOHD-NI01_2.pdf</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>6820-R2-67181-05</t>
+          <t>6820-R2-67065-07</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>14-PIT-79370</t>
+          <t>14-TE-68432</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>14-PIT-79370</t>
+          <t>14-TE-68432</t>
         </is>
       </c>
       <c r="G17" t="n">
@@ -996,30 +996,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6820-R2-67184-01_SIPG-CS01_1.pdf</t>
+          <t>6820-R2-67065-09-NOHD-NI01_1..pdf</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>6820-R2-67184-01</t>
+          <t>6820-R2-67065-09</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>14-TE-68150</t>
+          <t>14-LV-68260</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>14-TE-68150</t>
+          <t>14-LV-68260</t>
         </is>
       </c>
       <c r="G18" t="n">
@@ -1029,12 +1029,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>6820-R2-67184-03_SIPG-CS01_1..pdf</t>
+          <t>6820-R2-67065-09-NOHD-NI01_1.pdf</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6820-R2-67184-03</t>
+          <t>6820-R2-67065-09</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1042,17 +1042,17 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>14-FE-68150</t>
+          <t>14-LV-68260</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>14-FE-68150</t>
+          <t>14-LV-68260</t>
         </is>
       </c>
       <c r="G19" t="n">
@@ -1062,30 +1062,30 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6820-R2-67184-03_SIPG-CS01_1..pdf</t>
+          <t>6820-R2-67069-05_NOHD-NI01_0.pdf</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>6820-R2-67184-03</t>
+          <t>6820-R2-67069-05</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>14-FIT-68150</t>
+          <t>14-TE-68469</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>14-FIT-68150</t>
+          <t>14-TE-68469</t>
         </is>
       </c>
       <c r="G20" t="n">
@@ -1095,30 +1095,30 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>6820-R2-67184-05_SIPG-CS01_0.pdf</t>
+          <t>6820-R2-67072-03_NOHD-NI03_1.pdf</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>6820-R2-67184-05</t>
+          <t>6820-R2-67072-03</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>14-FV-68150</t>
+          <t>14-TI-68629</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>14-FV-68150</t>
+          <t>14-TI-68629</t>
         </is>
       </c>
       <c r="G21" t="n">
@@ -1128,30 +1128,30 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>6820-R2-67184-08_SIPG-CS01_0.pdf</t>
+          <t>6820-R2-67073-02_NOHD-SS01_0.pdf</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>6820-R2-67184-08</t>
+          <t>6820-R2-67073-02</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>14-TE-68421</t>
+          <t>14-HV-68460</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>14-TE-68421</t>
+          <t>14-HV-68460</t>
         </is>
       </c>
       <c r="G22" t="n">
@@ -1161,30 +1161,30 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>6820-R2-67214-01_CTWL-CS01_0..pdf</t>
+          <t>6820-R2-67076-04_SCXL-CS02_DELETED_1.pdf</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>6820-R2-67214-01</t>
+          <t>6820-R2-67076-04</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>14-LIT-68290</t>
+          <t>14-LV-68200</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>14-LIT-68290</t>
+          <t>14-LV-68200</t>
         </is>
       </c>
       <c r="G23" t="n">
@@ -1194,30 +1194,30 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>6820-R2-67271-02_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67076-05_SCXL-CS02_DELETED_1.pdf</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>6820-R2-67271-02</t>
+          <t>6820-R2-67076-05</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>14-LT-68240B</t>
+          <t>14-XV-68510</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>14-LT-68240B</t>
+          <t>14-XV-68510</t>
         </is>
       </c>
       <c r="G24" t="n">
@@ -1227,30 +1227,30 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>6820-R2-67271-03_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67080-01_SCXL-CS02_1..pdf</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>6820-R2-67271-03</t>
+          <t>6820-R2-67080-01</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>14-LIT-68240B</t>
+          <t>14-HV-68520</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>14-LIT-68240B</t>
+          <t>14-HV-68520</t>
         </is>
       </c>
       <c r="G25" t="n">
@@ -1260,30 +1260,30 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>6820-R2-67271-04_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67088-02_EPCW-CS01_1.pdf</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>6820-R2-67271-04</t>
+          <t>6820-R2-67088-02</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>14-LT-68240A</t>
+          <t>14-TI-68479</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>14-LT-68240A</t>
+          <t>14-TI-68479</t>
         </is>
       </c>
       <c r="G26" t="n">
@@ -1293,30 +1293,30 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>6820-R2-67271-05_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67093-02_NOHD-SS01_1.pdf</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6820-R2-67271-05</t>
+          <t>6820-R2-67093-02</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>14-LIT-68240A</t>
+          <t>14-FIT-68160</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>14-LIT-68240A</t>
+          <t>14-FIT-68160</t>
         </is>
       </c>
       <c r="G27" t="n">
@@ -1326,30 +1326,30 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>6820-R2-67278-02_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67093-02_NOHD-SS01_1.pdf</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6820-R2-67278-02</t>
+          <t>6820-R2-67093-02</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>14-LIT-68250B</t>
+          <t>14-TE-68433</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>14-LIT-68250B</t>
+          <t>14-TE-68433</t>
         </is>
       </c>
       <c r="G28" t="n">
@@ -1359,30 +1359,30 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>6820-R2-67278-03_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67093-04_NOHD-SS01_0.pdf</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>6820-R2-67278-03</t>
+          <t>6820-R2-67093-04</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>14-LT-68250B</t>
+          <t>14-LV-68270</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>14-LT-68250B</t>
+          <t>14-LV-68270</t>
         </is>
       </c>
       <c r="G29" t="n">
@@ -1392,30 +1392,30 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>6820-R2-67278-04_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67099-03_NOHD-CS01_0..pdf</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>6820-R2-67278-04</t>
+          <t>6820-R2-67099-03</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>10X8</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>14-LT-68250A</t>
+          <t>14-PSV-68399</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>14-LT-68250A</t>
+          <t>14-PSV-68399</t>
         </is>
       </c>
       <c r="G30" t="n">
@@ -1425,30 +1425,30 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>6820-R2-67285-02_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67107-05_SCXL-CS02_0..pdf</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>6820-R2-67285-02</t>
+          <t>6820-R2-67107-05</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>14-LT-68260B</t>
+          <t>14-FI-68159</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>14-LT-68260B</t>
+          <t>14-FI-68159</t>
         </is>
       </c>
       <c r="G31" t="n">
@@ -1458,30 +1458,30 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>6820-R2-67285-03_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67107-06_SCXL-CS02_0..pdf</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>6820-R2-67285-03</t>
+          <t>6820-R2-67107-06</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>14-LIT-68260B</t>
+          <t>14-TDV-68420</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>14-LIT-68260B</t>
+          <t>14-TDV-68420</t>
         </is>
       </c>
       <c r="G32" t="n">
@@ -1491,30 +1491,30 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>6820-R2-67285-04_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67107-06_SCXL-CS02_0..pdf</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>6820-R2-67285-04</t>
+          <t>6820-R2-67107-06</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>14-LT-68260A</t>
+          <t>14-PI-68639</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>14-LT-68260A</t>
+          <t>14-PI-68639</t>
         </is>
       </c>
       <c r="G33" t="n">
@@ -1524,30 +1524,30 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>6820-R2-67285-05_NOHD-NI01_0..pdf</t>
+          <t>6820-R2-67110-01_SIPG-CS01_0..pdf</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>6820-R2-67285-05</t>
+          <t>6820-R2-67110-01</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>14-LIT-68260A</t>
+          <t>VG-4</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>14-LIT-68260A</t>
+          <t>VG-4</t>
         </is>
       </c>
       <c r="G34" t="n">
@@ -1557,30 +1557,30 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>6820-R2-67293-02_NOHD-SS01_0..pdf</t>
+          <t>6820-R2-67110-01_SIPG-CS01_0..pdf</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>6820-R2-67293-02</t>
+          <t>6820-R2-67110-01</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1/2</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>14-LT-68270A</t>
+          <t>VG-7</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>14-LT-68270A</t>
+          <t>VG-7</t>
         </is>
       </c>
       <c r="G35" t="n">
@@ -1590,30 +1590,30 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>6820-R2-67293-03_NOHD-SS01_0..pdf</t>
+          <t>6820-R2-67111-03_EPCW-CS01_0..pdf</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>6820-R2-67293-03</t>
+          <t>6820-R2-67111-03</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>14-LIT-68270B</t>
+          <t>14-PV-68353</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>14-LIT-68270B</t>
+          <t>14-PV-68353</t>
         </is>
       </c>
       <c r="G36" t="n">
@@ -1623,30 +1623,30 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>6820-R2-67293-05_NOHD-SS01_0..pdf</t>
+          <t>6820-R2-67114-02_CTWL-CS01_1.pdf</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>6820-R2-67293-05</t>
+          <t>6820-R2-67114-02</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>14-LT-68270B</t>
+          <t>14-TI-68499</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>14-LT-68270B</t>
+          <t>14-TI-68499</t>
         </is>
       </c>
       <c r="G37" t="n">
@@ -1656,30 +1656,30 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>6820-R2-67351-01_NOHD-CS01_0..pdf</t>
+          <t>6820-R2-67115-02_CTWL-CS01_1.pdf</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>6820-R2-67351-01</t>
+          <t>6820-R2-67115-02</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>1.1/2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>14-PSE-68399</t>
+          <t>14-TI-68489</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>14-PSE-68399</t>
+          <t>14-TI-68489</t>
         </is>
       </c>
       <c r="G38" t="n">
@@ -1689,33 +1689,3123 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>6820-R2-67120-03_EPCW-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>6820-R2-67120-03</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>6</v>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>14-PI-68679</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>14-PI-68679</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>6820-R2-67121-02_CTWL-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>6820-R2-67121-02</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>15</v>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>14-TI-68929</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>14-TI-68929</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>6820-R2-67121-04_CTWL-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>6820-R2-67121-04</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>6</v>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>14-PI-68699</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>14-PI-68699</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>6820-R2-67122-02_NOHD-NI03_0.pdf</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>6820-R2-67122-02</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>16</v>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>14-TV-68450</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>14-TV-68450</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>6820-R2-67125-03_NOHD-SS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>6820-R2-67125-03</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>16</v>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>14-TE-68450</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>14-TE-68450</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>6820-R2-67125-04_NOHD-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>6820-R2-67125-04</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>18</v>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>14-FE-68180</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>14-FE-68180</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>6820-R2-67125-05_NOHD-SS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>6820-R2-67125-05</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>9</v>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>14-FV-68180</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>14-FV-68180</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>6820-R2-67129-06_EPCL-SS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>6820-R2-67129-06</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>7</v>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>14-PI-68829</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>14-PI-68829</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>6820-R2-67130-06_EPCL-SS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>6820-R2-67130-06</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>12</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>14-LV-68280</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>14-LV-68280</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>6820-R2-67130-09_EPCL-SS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>6820-R2-67130-09</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>7</v>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>14-PI-68819</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>14-PI-68819</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>6820-R2-67133-02_EPCL-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>6820-R2-67133-02</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>11</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>14-AE-68090</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>14-AE-68090</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>6820-R2-67134-03_EPCL-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>6820-R2-67134-03</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>6</v>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>14-FI-68119</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>14-FI-68119</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>6820-R2-67139-05_CTWL-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>6820-R2-67139-05</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>7</v>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>14-PI-68849</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>14-PI-68849</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>6820-R2-67140-06_CTWL-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>6820-R2-67140-06</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>6</v>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>14-LV-68290</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>14-LV-68290</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>6820-R2-67140-09_CTWL-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>6820-R2-67140-09</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>7</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>14-PI-68839</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>14-PI-68839</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>6820-R2-67143-01_NOHD-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>6820-R2-67143-01</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>10</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>14-PIT-68353</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>14-PIT-68353</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>6820-R2-67146-02_EPCL-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>6820-R2-67146-02</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>13</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>14-PIT-68370A</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>14-PIT-68370A</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>6820-R2-67146-02_EPCL-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>6820-R2-67146-02</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>14</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>14-PIT-68370B</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>14-PIT-68370B</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>6820-R2-67164-02_CTWL-CS01_2.pdf</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>6820-R2-67164-02</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>16</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>14-FE-68170</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>14-FE-68170</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>6820-R2-67164-03_CTWL-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>6820-R2-67164-03</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>12</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>14-TI-68709</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>14-TI-68709</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>6820-R2-67165-03_POWL-XX01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>6820-R2-67165-03</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>11</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>PIT-68300</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>PIT-68300</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>6820-R2-67181-02_SLPG-CS01_1..pdf</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>6820-R2-67181-02</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>12</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>07-PV-79370</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>07-PV-79370</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>6820-R2-67181-05_SLPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>6820-R2-67181-05</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>13</v>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>14-PIT-79370</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>14-PIT-79370</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>6820-R2-67181-06_SLPG-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>6820-R2-67181-06</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>9</v>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>14-PI-68869</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>14-PI-68869</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-01_SIPG-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-01</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>15</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-01_SIPG-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-01</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>16</v>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>14-TE-68150</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>14-TE-68150</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02_SIPG-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" t="inlineStr"/>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02_SIPG-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02</t>
+        </is>
+      </c>
+      <c r="C66" t="n">
+        <v>13</v>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02_SIPG-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>15</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>14-PIT-68150</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>14-PIT-68150</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02_SIPG-CS01_1.pdf</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-02</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>16</v>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>14-FIT-68150</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>14-FIT-68150</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03_SIPG-CS01_1..pdf</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" t="inlineStr"/>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03_SIPG-CS01_1..pdf</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>14</v>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03_SIPG-CS01_1..pdf</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>17</v>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>14-FE-68150</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>14-FE-68150</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03_SIPG-CS01_1..pdf</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-03</t>
+        </is>
+      </c>
+      <c r="C72" t="n">
+        <v>18</v>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>14-FIT-68150</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>14-FIT-68150</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-05_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-05</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>14-FV-68150</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>14-FV-68150</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-06_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-06</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>9</v>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-07_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-07</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>14</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-07_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-07</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>15</v>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>6X1</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>SP-6875</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>SP-6875</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-08_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-08</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>13</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>14-TE-68421</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>14-TE-68421</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-09_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-09</t>
+        </is>
+      </c>
+      <c r="C78" t="n">
+        <v>7</v>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-12_SIPG-CS01_1..pdf</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>6820-R2-67184-12</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>11</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-01_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-01</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>7</v>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-02_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-02</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>14</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>1/2</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-03_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-03</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>10</v>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-03_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-03</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>11</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>14-PI-68899</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>14-PI-68899</t>
+        </is>
+      </c>
+      <c r="G83" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-04_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>6820-R2-67189-04</t>
+        </is>
+      </c>
+      <c r="C84" t="n">
+        <v>7</v>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G84" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>6820-R2-67213-02_NOHD-SS03_0.pdf</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>6820-R2-67213-02</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>9</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>SP-6841</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>SP-6841</t>
+        </is>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>6820-R2-67214-01_CTWL-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>6820-R2-67214-01</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>5</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>14-LIT-68290</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>14-LIT-68290</t>
+        </is>
+      </c>
+      <c r="G86" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>6820-R2-67221-03_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>6820-R2-67221-03</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>12</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>VG-4</t>
+        </is>
+      </c>
+      <c r="G87" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>6820-R2-67221-03_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>6820-R2-67221-03</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>13</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G88" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>6820-R2-67221-03_SIPG-CS01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>6820-R2-67221-03</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>14</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>14-PI-68859</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>14-PI-68859</t>
+        </is>
+      </c>
+      <c r="G89" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>6820-R2-67222-03_EPCL-SS01_1..pdf</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>6820-R2-67222-03</t>
+        </is>
+      </c>
+      <c r="C90" t="n">
+        <v>9</v>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>14-FIT-68190</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>14-FIT-68190</t>
+        </is>
+      </c>
+      <c r="G90" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>6820-R2-67225-03_SLPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>6820-R2-67225-03</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>8</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>10X8</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>14-PSV-68919A</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>14-PSV-68919A</t>
+        </is>
+      </c>
+      <c r="G91" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>6820-R2-67229-02_SCXL-CS02_0..pdf</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>6820-R2-67229-02</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>14</v>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>14-PI-68769</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>14-PI-68769</t>
+        </is>
+      </c>
+      <c r="G92" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-02_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-02</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>5</v>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>14-LT-68240B</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>14-LT-68240B</t>
+        </is>
+      </c>
+      <c r="G93" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-03_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-03</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>8</v>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>14-LIT-68240B</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>14-LIT-68240B</t>
+        </is>
+      </c>
+      <c r="G94" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-04_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-04</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>5</v>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>14-LT-68240A</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>14-LT-68240A</t>
+        </is>
+      </c>
+      <c r="G95" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-05_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>6820-R2-67271-05</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>8</v>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>14-LIT-68240A</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>14-LIT-68240A</t>
+        </is>
+      </c>
+      <c r="G96" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>6820-R2-67272-01_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>6820-R2-67272-01</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>12</v>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>14-PIT-68351</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>14-PIT-68351</t>
+        </is>
+      </c>
+      <c r="G97" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>6820-R2-67274-01_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>6820-R2-67274-01</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>3</v>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>14-TE-68411</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>14-TE-68411</t>
+        </is>
+      </c>
+      <c r="G98" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>6820-R2-67275-05_SCXL-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>6820-R2-67275-05</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>4</v>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>14-LIT-68200</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>14-LIT-68200</t>
+        </is>
+      </c>
+      <c r="G99" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>6820-R2-67275-06_SCXL-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>6820-R2-67275-06</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>4</v>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>14-LIT-68200</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>14-LIT-68200</t>
+        </is>
+      </c>
+      <c r="G100" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>6820-R2-67278-02_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>6820-R2-67278-02</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>4</v>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>14-LIT-68250B</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>14-LIT-68250B</t>
+        </is>
+      </c>
+      <c r="G101" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>6820-R2-67278-03_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>6820-R2-67278-03</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>5</v>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>14-LT-68250B</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>14-LT-68250B</t>
+        </is>
+      </c>
+      <c r="G102" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>6820-R2-67278-04_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>6820-R2-67278-04</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>5</v>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>14-LT-68250A</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>14-LT-68250A</t>
+        </is>
+      </c>
+      <c r="G103" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>6820-R2-67284-01_EPCW-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>6820-R2-67284-01</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>8</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>14-PIT-68342</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>14-PIT-68342</t>
+        </is>
+      </c>
+      <c r="G104" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-02_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-02</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>5</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>14-LT-68260B</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>14-LT-68260B</t>
+        </is>
+      </c>
+      <c r="G105" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-03_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-03</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>8</v>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>14-LIT-68260B</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>14-LIT-68260B</t>
+        </is>
+      </c>
+      <c r="G106" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-04_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-04</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>5</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>14-LT-68260A</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>14-LT-68260A</t>
+        </is>
+      </c>
+      <c r="G107" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-05_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>6820-R2-67285-05</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>8</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>14-LIT-68260A</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>14-LIT-68260A</t>
+        </is>
+      </c>
+      <c r="G108" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>6820-R2-67286-01_NOHD-NI01_0.pdf</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>6820-R2-67286-01</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>11</v>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>14-PIT-68352</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>14-PIT-68352</t>
+        </is>
+      </c>
+      <c r="G109" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>6820-R2-67287-03_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>6820-R2-67287-03</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>3</v>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>14-TE-68412</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>14-TE-68412</t>
+        </is>
+      </c>
+      <c r="G110" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>6820-R2-67292-01_EPCW-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>6820-R2-67292-01</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>8</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>14-PIT-68343</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>14-PIT-68343</t>
+        </is>
+      </c>
+      <c r="G111" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-02_NOHD-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-02</t>
+        </is>
+      </c>
+      <c r="C112" t="n">
+        <v>5</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>14-LT-68270A</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>14-LT-68270A</t>
+        </is>
+      </c>
+      <c r="G112" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-03_NOHD-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-03</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>9</v>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>14-LIT-68270B</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>14-LIT-68270B</t>
+        </is>
+      </c>
+      <c r="G113" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-04_NOHD-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-04</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>9</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>14-LIT-68270A</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>14-LIT-68270A</t>
+        </is>
+      </c>
+      <c r="G114" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-05_NOHD-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>6820-R2-67293-05</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>5</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>14-LT-68270B</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>14-LT-68270B</t>
+        </is>
+      </c>
+      <c r="G115" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>6820-R2-67294-03_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>6820-R2-67294-03</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>3</v>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>14-TE-68413</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>14-TE-68413</t>
+        </is>
+      </c>
+      <c r="G116" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>6820-R2-67296-05_EPCL-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>6820-R2-67296-05</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>4</v>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>14-LIT-68280</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>14-LIT-68280</t>
+        </is>
+      </c>
+      <c r="G117" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>6820-R2-67296-06_EPCL-SS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>6820-R2-67296-06</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>4</v>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>14-LIT-68280</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>14-LIT-68280</t>
+        </is>
+      </c>
+      <c r="G118" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>6820-R2-67318-02_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>6820-R2-67318-02</t>
+        </is>
+      </c>
+      <c r="C119" t="n">
+        <v>9</v>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>10X6</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>14-PSV-68909B</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>14-PSV-68909B</t>
+        </is>
+      </c>
+      <c r="G119" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>6820-R2-67320-02_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>6820-R2-67320-02</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>9</v>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>10X6</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>14-PSV-68909A</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>14-PSV-68909A</t>
+        </is>
+      </c>
+      <c r="G120" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>6820-R2-67321-01_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>6820-R2-67321-01</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>13</v>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>1X3/4</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>14-PSV-68359</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>14-PSV-68359</t>
+        </is>
+      </c>
+      <c r="G121" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>6820-R2-67322-01_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>6820-R2-67322-01</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>17</v>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>2X1</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>14-PSV-68719</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>14-PSV-68719</t>
+        </is>
+      </c>
+      <c r="G122" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>6820-R2-67323-01_NOHD-NI01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>6820-R2-67323-01</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>13</v>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>1X3/4</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>14-PSV-68729</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>14-PSV-68729</t>
+        </is>
+      </c>
+      <c r="G123" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>6820-R2-67351-01_NOHD-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>6820-R2-67351-01</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>7</v>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>14-PSE-68399</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>14-PSE-68399</t>
+        </is>
+      </c>
+      <c r="G124" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
           <t>6820-R2-67361-02_SCXL-CS02_1..pdf</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B125" t="inlineStr">
         <is>
           <t>6820-R2-67361-02</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="C125" t="n">
         <v>17</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D125" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E125" t="inlineStr">
         <is>
           <t>14-AE-68001</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F125" t="inlineStr">
         <is>
           <t>14-AE-68001</t>
         </is>
       </c>
-      <c r="G39" t="n">
+      <c r="G125" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>6820-R2-67361-04_SCXL-CS02_0..pdf</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>6820-R2-67361-04</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>16</v>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>14-LV-68200</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>14-LV-68200</t>
+        </is>
+      </c>
+      <c r="G126" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>6820-R2-67361-05_SCXL-CS02_1..pdf</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>6820-R2-67361-05</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>15</v>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>14-HV-68510</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>14-HV-68510</t>
+        </is>
+      </c>
+      <c r="G127" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>6820-R2-67367-03_SLPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>6820-R2-67367-03</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>8</v>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>10X8</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>14-PSV-68919B</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>14-PSV-68919B</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>6820-R2-67375-01_EPCW-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>6820-R2-67375-01</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>3</v>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>14-TE-68423</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>14-TE-68423</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>6820-R2-67377-01_SLPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>6820-R2-67377-01</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>3</v>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>14-TE-68422</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>14-TE-68422</t>
+        </is>
+      </c>
+      <c r="G130" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>6820-R2-67380-03_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>6820-R2-67380-03</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>6</v>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G131" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>6820-R2-67380-04_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>6820-R2-67380-04</t>
+        </is>
+      </c>
+      <c r="C132" t="n">
+        <v>6</v>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>3/4</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>VG-7</t>
+        </is>
+      </c>
+      <c r="G132" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>6820-R2-67382-01_SIPG-CS01_0..pdf</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>6820-R2-67382-01</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>9</v>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>1.1/2</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>14-PIT-68341</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>14-PIT-68341</t>
+        </is>
+      </c>
+      <c r="G133" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>